<commit_message>
renaming the excel columns
</commit_message>
<xml_diff>
--- a/public/templates/coo_org_chart_template.xlsx
+++ b/public/templates/coo_org_chart_template.xlsx
@@ -22,10 +22,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="28">
   <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parent ID</t>
+    <t xml:space="preserve">Sr No.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sr No. to report to</t>
   </si>
   <si>
     <t xml:space="preserve">Role</t>
@@ -467,8 +467,8 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>

</xml_diff>